<commit_message>
add sheet reading (groery comparison)
</commit_message>
<xml_diff>
--- a/prixEpicerie.xlsx
+++ b/prixEpicerie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dalto\OneDrive\Documents\Ecole\Programmation1\Team_Rosemarie_and_Leo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E56AF55-3844-4521-8808-E64B4A77CDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C3835DE-4BCB-4244-97FE-2D970A25F201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{2198D66A-2FBF-4C5F-A307-23CE27175DD6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{2198D66A-2FBF-4C5F-A307-23CE27175DD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Metro" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
   <si>
     <t>Apple</t>
   </si>
@@ -478,7 +478,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -513,9 +513,50 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C57A07B-F668-49AB-9E14-5DC649963E41}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>